<commit_message>
Optimisation portfolio BTS: nettoyage CSS + refonte mode clair + dates 2026
</commit_message>
<xml_diff>
--- a/E5/annexe-bts_aziz.xlsx
+++ b/E5/annexe-bts_aziz.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\33658\Desktop\PortfolioAZiz\E5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62263C67-1B7A-497E-93CA-22F06240C124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{764F5240-ED8D-48A5-8195-F4E4FD0E3D55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="56">
   <si>
     <t>Gérer le patrimoine informatique</t>
   </si>
@@ -187,9 +187,6 @@
   </si>
   <si>
     <t>Support Helpdesk : Gestion des tickets d'assistance et résolution d'incidents utilisateurs</t>
-  </si>
-  <si>
-    <t>TP : Virtualisation &amp; Haute Disponibilité (Cluster Proxmox, Migration de VM)</t>
   </si>
   <si>
     <t>Période (sous la forme du 02/09/2024 au 09/03/2026)</t>
@@ -223,6 +220,9 @@
       </rPr>
       <t>ACL)</t>
     </r>
+  </si>
+  <si>
+    <t>TP : Installation de Proxmox VE et Mise en Œuvre d'un Cluster en Haute Disponibilité (Migration de VM)</t>
   </si>
 </sst>
 </file>
@@ -743,7 +743,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -802,6 +802,9 @@
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="29" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -881,12 +884,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1209,56 +1206,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="39.9" customHeight="1">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="23" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22" t="s">
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="H1" s="22"/>
+      <c r="H1" s="23"/>
     </row>
     <row r="2" spans="1:43" ht="41.1" customHeight="1" thickBot="1">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="23" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23"/>
     </row>
     <row r="3" spans="1:43" ht="39.9" customHeight="1">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="29" t="s">
+      <c r="B3" s="25"/>
+      <c r="C3" s="25"/>
+      <c r="D3" s="25"/>
+      <c r="E3" s="26"/>
+      <c r="F3" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="G3" s="24"/>
-      <c r="H3" s="30"/>
+      <c r="G3" s="25"/>
+      <c r="H3" s="31"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="39.9" customHeight="1">
-      <c r="A4" s="26" t="s">
+      <c r="A4" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="B4" s="27"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="28"/>
+      <c r="B4" s="28"/>
+      <c r="C4" s="28"/>
+      <c r="D4" s="28"/>
+      <c r="E4" s="29"/>
       <c r="F4" s="6" t="s">
         <v>8</v>
       </c>
@@ -1270,23 +1267,23 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="39.9" customHeight="1" thickBot="1">
-      <c r="A5" s="44" t="s">
+      <c r="A5" s="45" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="45"/>
-      <c r="C5" s="45"/>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="45"/>
-      <c r="H5" s="46"/>
+      <c r="B5" s="46"/>
+      <c r="C5" s="46"/>
+      <c r="D5" s="46"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="46"/>
+      <c r="G5" s="46"/>
+      <c r="H5" s="47"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1">
-      <c r="A6" s="37" t="s">
+      <c r="A6" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="B6" s="42" t="s">
-        <v>49</v>
+      <c r="B6" s="43" t="s">
+        <v>48</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>0</v>
@@ -1308,8 +1305,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="324.89999999999998" customHeight="1" thickBot="1">
-      <c r="A7" s="38"/>
-      <c r="B7" s="43"/>
+      <c r="A7" s="39"/>
+      <c r="B7" s="44"/>
       <c r="C7" s="9" t="s">
         <v>9</v>
       </c>
@@ -1365,16 +1362,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="72" customHeight="1" thickBot="1">
-      <c r="A8" s="39" t="s">
+      <c r="A8" s="40" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="41"/>
+      <c r="B8" s="41"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="41"/>
+      <c r="E8" s="41"/>
+      <c r="F8" s="41"/>
+      <c r="G8" s="41"/>
+      <c r="H8" s="42"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1476,9 +1473,7 @@
       <c r="C10" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="13" t="s">
-        <v>46</v>
-      </c>
+      <c r="D10" s="13"/>
       <c r="E10" s="13" t="s">
         <v>22</v>
       </c>
@@ -1527,7 +1522,7 @@
     </row>
     <row r="11" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" thickBot="1">
       <c r="A11" s="5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B11" s="15" t="s">
         <v>30</v>
@@ -1591,7 +1586,7 @@
         <v>22</v>
       </c>
       <c r="D12" s="13" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="E12" s="13"/>
       <c r="F12" s="13"/>
@@ -1637,9 +1632,9 @@
     </row>
     <row r="13" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" thickBot="1">
       <c r="A13" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="B13" s="48">
+        <v>50</v>
+      </c>
+      <c r="B13" s="20">
         <v>45939</v>
       </c>
       <c r="C13" s="13" t="s">
@@ -1647,7 +1642,7 @@
       </c>
       <c r="D13" s="13"/>
       <c r="E13" s="13"/>
-      <c r="F13" s="47"/>
+      <c r="F13" s="19"/>
       <c r="G13" s="13" t="s">
         <v>46</v>
       </c>
@@ -1745,10 +1740,10 @@
     </row>
     <row r="15" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" thickBot="1">
       <c r="A15" s="5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C15" s="13" t="s">
         <v>22</v>
@@ -1797,10 +1792,10 @@
     </row>
     <row r="16" spans="1:43" s="2" customFormat="1" ht="52.2" customHeight="1" thickBot="1">
       <c r="A16" s="5" t="s">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C16" s="14" t="s">
         <v>22</v>
@@ -1813,7 +1808,9 @@
       <c r="G16" s="14" t="s">
         <v>22</v>
       </c>
-      <c r="H16" s="14"/>
+      <c r="H16" s="14" t="s">
+        <v>46</v>
+      </c>
       <c r="I16"/>
       <c r="J16"/>
       <c r="K16"/>
@@ -1905,7 +1902,7 @@
     </row>
     <row r="18" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" thickBot="1">
       <c r="A18" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B18" s="17" t="s">
         <v>33</v>
@@ -1955,16 +1952,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" thickBot="1">
-      <c r="A19" s="31" t="s">
+      <c r="A19" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="B19" s="32"/>
-      <c r="C19" s="32"/>
-      <c r="D19" s="32"/>
-      <c r="E19" s="32"/>
-      <c r="F19" s="32"/>
-      <c r="G19" s="32"/>
-      <c r="H19" s="33"/>
+      <c r="B19" s="33"/>
+      <c r="C19" s="33"/>
+      <c r="D19" s="33"/>
+      <c r="E19" s="33"/>
+      <c r="F19" s="33"/>
+      <c r="G19" s="33"/>
+      <c r="H19" s="34"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -2005,7 +2002,7 @@
       <c r="A20" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="21" t="s">
         <v>26</v>
       </c>
       <c r="C20" s="13" t="s">
@@ -2058,7 +2055,7 @@
       <c r="A21" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="B21" s="21"/>
+      <c r="B21" s="22"/>
       <c r="C21" s="13" t="s">
         <v>22</v>
       </c>
@@ -2109,7 +2106,7 @@
       <c r="A22" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B22" s="21"/>
+      <c r="B22" s="22"/>
       <c r="C22" s="13" t="s">
         <v>22</v>
       </c>
@@ -2118,7 +2115,9 @@
       </c>
       <c r="E22" s="13"/>
       <c r="F22" s="13"/>
-      <c r="G22" s="13"/>
+      <c r="G22" s="13" t="s">
+        <v>46</v>
+      </c>
       <c r="H22" s="11"/>
       <c r="I22"/>
       <c r="J22"/>
@@ -2160,7 +2159,7 @@
       <c r="A23" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B23" s="21"/>
+      <c r="B23" s="22"/>
       <c r="C23" s="13"/>
       <c r="D23" s="13" t="s">
         <v>22</v>
@@ -2208,16 +2207,16 @@
       <c r="AQ23"/>
     </row>
     <row r="24" spans="1:43" s="2" customFormat="1" ht="39.9" customHeight="1" thickBot="1">
-      <c r="A24" s="34" t="s">
+      <c r="A24" s="35" t="s">
         <v>19</v>
       </c>
-      <c r="B24" s="35"/>
-      <c r="C24" s="35"/>
-      <c r="D24" s="35"/>
-      <c r="E24" s="35"/>
-      <c r="F24" s="35"/>
-      <c r="G24" s="35"/>
-      <c r="H24" s="36"/>
+      <c r="B24" s="36"/>
+      <c r="C24" s="36"/>
+      <c r="D24" s="36"/>
+      <c r="E24" s="36"/>
+      <c r="F24" s="36"/>
+      <c r="G24" s="36"/>
+      <c r="H24" s="37"/>
       <c r="I24"/>
       <c r="J24"/>
       <c r="K24"/>
@@ -2258,7 +2257,7 @@
       <c r="A25" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="B25" s="20" t="s">
+      <c r="B25" s="21" t="s">
         <v>26</v>
       </c>
       <c r="C25" s="12" t="s">
@@ -2313,7 +2312,7 @@
       <c r="A26" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B26" s="21"/>
+      <c r="B26" s="22"/>
       <c r="C26" s="12" t="s">
         <v>22</v>
       </c>
@@ -2329,7 +2328,7 @@
       <c r="A27" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="21"/>
+      <c r="B27" s="22"/>
       <c r="C27" s="12" t="s">
         <v>22</v>
       </c>
@@ -2347,7 +2346,7 @@
       <c r="A28" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="B28" s="21"/>
+      <c r="B28" s="22"/>
       <c r="C28" s="12"/>
       <c r="D28" s="12" t="s">
         <v>22</v>
@@ -2361,7 +2360,7 @@
     </row>
     <row r="29" spans="1:43" customFormat="1" ht="43.8" customHeight="1" thickBot="1">
       <c r="A29" s="11"/>
-      <c r="B29" s="21"/>
+      <c r="B29" s="22"/>
     </row>
     <row r="30" spans="1:43" customFormat="1"/>
     <row r="31" spans="1:43" customFormat="1"/>

</xml_diff>